<commit_message>
Fixed the Care room and it can now get hunggry
</commit_message>
<xml_diff>
--- a/job_plannar.xlsx
+++ b/job_plannar.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxwe\Desktop\Delta_Alpha_BOND_NEW\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7268B07F-813A-418C-9F2D-9206823D6B1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4422BF88-49E1-429A-B13A-8FCF4EAC6EBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-44370" yWindow="825" windowWidth="41445" windowHeight="18525" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15420" yWindow="2100" windowWidth="19575" windowHeight="18525" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1148" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1148" uniqueCount="268">
   <si>
     <t>Pittsburgh Job Search + Community Planner</t>
   </si>
@@ -914,6 +914,9 @@
   <si>
     <t>31
 Sun: weekly reset only</t>
+  </si>
+  <si>
+    <t>Done</t>
   </si>
 </sst>
 </file>
@@ -923,7 +926,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -955,8 +958,13 @@
       <color rgb="FF1F2937"/>
       <name val="Carlito"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Carlito"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -991,6 +999,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFAFAFA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1090,7 +1110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1170,11 +1190,10 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1185,9 +1204,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1216,10 +1232,26 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1537,16 +1569,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="32"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="31"/>
     </row>
     <row r="3" spans="1:8" ht="21.95" customHeight="1">
       <c r="A3" s="1" t="s">
@@ -1699,13 +1731,13 @@
         <f>COUNTA(Plan_90D!A4:A500)</f>
         <v>80</v>
       </c>
-      <c r="D13" s="40" t="s">
+      <c r="D13" s="38" t="s">
         <v>32</v>
       </c>
-      <c r="E13" s="41"/>
-      <c r="F13" s="41"/>
-      <c r="G13" s="41"/>
-      <c r="H13" s="42"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="39"/>
+      <c r="H13" s="40"/>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1">
       <c r="A14" s="5" t="s">
@@ -1713,15 +1745,15 @@
       </c>
       <c r="B14" s="6">
         <f>COUNTIF(Plan_90D!L4:L500,"Done")</f>
-        <v>0</v>
-      </c>
-      <c r="D14" s="34" t="s">
+        <v>2</v>
+      </c>
+      <c r="D14" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="E14" s="35"/>
-      <c r="F14" s="35"/>
-      <c r="G14" s="35"/>
-      <c r="H14" s="36"/>
+      <c r="E14" s="33"/>
+      <c r="F14" s="33"/>
+      <c r="G14" s="33"/>
+      <c r="H14" s="34"/>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1">
       <c r="A15" s="5" t="s">
@@ -1729,15 +1761,15 @@
       </c>
       <c r="B15" s="9">
         <f>IFERROR(B14/B13,0)</f>
-        <v>0</v>
-      </c>
-      <c r="D15" s="34" t="s">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="D15" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="E15" s="35"/>
-      <c r="F15" s="35"/>
-      <c r="G15" s="35"/>
-      <c r="H15" s="36"/>
+      <c r="E15" s="33"/>
+      <c r="F15" s="33"/>
+      <c r="G15" s="33"/>
+      <c r="H15" s="34"/>
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1">
       <c r="A16" s="5" t="s">
@@ -1747,13 +1779,13 @@
         <f>COUNTA(Weekly_Plan!A4:A100)</f>
         <v>16</v>
       </c>
-      <c r="D16" s="34" t="s">
+      <c r="D16" s="32" t="s">
         <v>38</v>
       </c>
-      <c r="E16" s="35"/>
-      <c r="F16" s="35"/>
-      <c r="G16" s="35"/>
-      <c r="H16" s="36"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="34"/>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1">
       <c r="A17" s="7" t="s">
@@ -1763,22 +1795,22 @@
         <f>COUNTIF(Weekly_Plan!E4:E100,"Done")</f>
         <v>0</v>
       </c>
-      <c r="D17" s="34" t="s">
+      <c r="D17" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="E17" s="35"/>
-      <c r="F17" s="35"/>
-      <c r="G17" s="35"/>
-      <c r="H17" s="36"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="33"/>
+      <c r="H17" s="34"/>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1">
-      <c r="D18" s="37" t="s">
+      <c r="D18" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="E18" s="38"/>
-      <c r="F18" s="38"/>
-      <c r="G18" s="38"/>
-      <c r="H18" s="39"/>
+      <c r="E18" s="36"/>
+      <c r="F18" s="36"/>
+      <c r="G18" s="36"/>
+      <c r="H18" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -1809,15 +1841,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="26.1" customHeight="1">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="32"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="31"/>
     </row>
     <row r="3" spans="1:7" ht="15">
       <c r="A3" s="13" t="s">
@@ -2089,14 +2121,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.1" customHeight="1">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="29" t="s">
         <v>104</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="32"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="31"/>
     </row>
     <row r="3" spans="1:6" ht="15">
       <c r="A3" s="13" t="s">
@@ -2449,21 +2481,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="26.1" customHeight="1">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="29" t="s">
         <v>142</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-      <c r="K1" s="31"/>
-      <c r="L1" s="31"/>
-      <c r="M1" s="32"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="31"/>
     </row>
     <row r="3" spans="1:13" ht="15">
       <c r="A3" s="13" t="s">
@@ -2513,190 +2545,190 @@
       <c r="B4" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="45" t="s">
         <v>155</v>
       </c>
-      <c r="D4" s="10" t="s">
-        <v>156</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="F4" s="10" t="s">
+      <c r="D4" s="45" t="s">
+        <v>156</v>
+      </c>
+      <c r="E4" s="46" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" s="45" t="s">
         <v>157</v>
       </c>
-      <c r="G4" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="H4" s="10" t="s">
+      <c r="G4" s="45" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="45" t="s">
         <v>158</v>
       </c>
-      <c r="I4" s="10" t="s">
-        <v>159</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>160</v>
-      </c>
-      <c r="K4" s="10" t="s">
+      <c r="I4" s="45" t="s">
+        <v>159</v>
+      </c>
+      <c r="J4" s="45" t="s">
+        <v>160</v>
+      </c>
+      <c r="K4" s="45" t="s">
         <v>161</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>56</v>
+        <v>267</v>
       </c>
       <c r="M4" s="4"/>
     </row>
     <row r="5" spans="1:13" ht="54">
-      <c r="A5" s="43">
+      <c r="A5" s="27">
         <v>46133</v>
       </c>
-      <c r="B5" s="44" t="s">
+      <c r="B5" s="28" t="s">
         <v>162</v>
       </c>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="47" t="s">
         <v>155</v>
       </c>
-      <c r="D5" s="44" t="s">
-        <v>156</v>
-      </c>
-      <c r="E5" s="44" t="s">
-        <v>5</v>
-      </c>
-      <c r="F5" s="44" t="s">
+      <c r="D5" s="47" t="s">
+        <v>156</v>
+      </c>
+      <c r="E5" s="48" t="s">
+        <v>5</v>
+      </c>
+      <c r="F5" s="47" t="s">
         <v>163</v>
       </c>
-      <c r="G5" s="44" t="s">
-        <v>25</v>
-      </c>
-      <c r="H5" s="44" t="s">
+      <c r="G5" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" s="47" t="s">
         <v>164</v>
       </c>
-      <c r="I5" s="44" t="s">
-        <v>159</v>
-      </c>
-      <c r="J5" s="44" t="s">
-        <v>160</v>
-      </c>
-      <c r="K5" s="44" t="s">
+      <c r="I5" s="47" t="s">
+        <v>159</v>
+      </c>
+      <c r="J5" s="47" t="s">
+        <v>160</v>
+      </c>
+      <c r="K5" s="47" t="s">
         <v>165</v>
       </c>
-      <c r="L5" s="44" t="s">
-        <v>56</v>
+      <c r="L5" s="47" t="s">
+        <v>267</v>
       </c>
       <c r="M5" s="6"/>
     </row>
     <row r="6" spans="1:13" ht="54">
-      <c r="A6" s="43">
+      <c r="A6" s="27">
         <v>46134</v>
       </c>
-      <c r="B6" s="44" t="s">
+      <c r="B6" s="28" t="s">
         <v>166</v>
       </c>
-      <c r="C6" s="44" t="s">
+      <c r="C6" s="28" t="s">
         <v>155</v>
       </c>
-      <c r="D6" s="44" t="s">
-        <v>156</v>
-      </c>
-      <c r="E6" s="44" t="s">
-        <v>5</v>
-      </c>
-      <c r="F6" s="44" t="s">
+      <c r="D6" s="28" t="s">
+        <v>156</v>
+      </c>
+      <c r="E6" s="28" t="s">
+        <v>5</v>
+      </c>
+      <c r="F6" s="28" t="s">
         <v>167</v>
       </c>
-      <c r="G6" s="44" t="s">
-        <v>25</v>
-      </c>
-      <c r="H6" s="44" t="s">
+      <c r="G6" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6" s="28" t="s">
         <v>168</v>
       </c>
-      <c r="I6" s="44" t="s">
-        <v>159</v>
-      </c>
-      <c r="J6" s="44" t="s">
-        <v>160</v>
-      </c>
-      <c r="K6" s="44" t="s">
+      <c r="I6" s="28" t="s">
+        <v>159</v>
+      </c>
+      <c r="J6" s="28" t="s">
+        <v>160</v>
+      </c>
+      <c r="K6" s="28" t="s">
         <v>169</v>
       </c>
-      <c r="L6" s="44" t="s">
+      <c r="L6" s="28" t="s">
         <v>56</v>
       </c>
       <c r="M6" s="6"/>
     </row>
     <row r="7" spans="1:13" ht="72">
-      <c r="A7" s="43">
+      <c r="A7" s="27">
         <v>46135</v>
       </c>
-      <c r="B7" s="44" t="s">
+      <c r="B7" s="28" t="s">
         <v>170</v>
       </c>
-      <c r="C7" s="44" t="s">
+      <c r="C7" s="28" t="s">
         <v>155</v>
       </c>
-      <c r="D7" s="44" t="s">
-        <v>156</v>
-      </c>
-      <c r="E7" s="44" t="s">
-        <v>5</v>
-      </c>
-      <c r="F7" s="44" t="s">
+      <c r="D7" s="28" t="s">
+        <v>156</v>
+      </c>
+      <c r="E7" s="28" t="s">
+        <v>5</v>
+      </c>
+      <c r="F7" s="28" t="s">
         <v>171</v>
       </c>
-      <c r="G7" s="44" t="s">
-        <v>25</v>
-      </c>
-      <c r="H7" s="44" t="s">
+      <c r="G7" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" s="28" t="s">
         <v>172</v>
       </c>
-      <c r="I7" s="44" t="s">
-        <v>159</v>
-      </c>
-      <c r="J7" s="44" t="s">
-        <v>160</v>
-      </c>
-      <c r="K7" s="44" t="s">
+      <c r="I7" s="28" t="s">
+        <v>159</v>
+      </c>
+      <c r="J7" s="28" t="s">
+        <v>160</v>
+      </c>
+      <c r="K7" s="28" t="s">
         <v>173</v>
       </c>
-      <c r="L7" s="44" t="s">
+      <c r="L7" s="28" t="s">
         <v>56</v>
       </c>
       <c r="M7" s="6"/>
     </row>
     <row r="8" spans="1:13" ht="54">
-      <c r="A8" s="43">
+      <c r="A8" s="27">
         <v>46136</v>
       </c>
-      <c r="B8" s="44" t="s">
+      <c r="B8" s="28" t="s">
         <v>174</v>
       </c>
-      <c r="C8" s="44" t="s">
+      <c r="C8" s="28" t="s">
         <v>155</v>
       </c>
-      <c r="D8" s="44" t="s">
-        <v>156</v>
-      </c>
-      <c r="E8" s="44" t="s">
-        <v>5</v>
-      </c>
-      <c r="F8" s="44" t="s">
+      <c r="D8" s="28" t="s">
+        <v>156</v>
+      </c>
+      <c r="E8" s="28" t="s">
+        <v>5</v>
+      </c>
+      <c r="F8" s="28" t="s">
         <v>175</v>
       </c>
-      <c r="G8" s="44" t="s">
-        <v>25</v>
-      </c>
-      <c r="H8" s="44" t="s">
+      <c r="G8" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" s="28" t="s">
         <v>176</v>
       </c>
-      <c r="I8" s="44" t="s">
+      <c r="I8" s="28" t="s">
         <v>177</v>
       </c>
-      <c r="J8" s="44" t="s">
-        <v>160</v>
-      </c>
-      <c r="K8" s="44" t="s">
+      <c r="J8" s="28" t="s">
+        <v>160</v>
+      </c>
+      <c r="K8" s="28" t="s">
         <v>178</v>
       </c>
-      <c r="L8" s="44" t="s">
+      <c r="L8" s="28" t="s">
         <v>56</v>
       </c>
       <c r="M8" s="6"/>
@@ -5666,15 +5698,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="29" t="s">
         <v>194</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="32"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="31"/>
     </row>
     <row r="3" spans="1:7" ht="15">
       <c r="A3" s="13" t="s">
@@ -5700,175 +5732,181 @@
       </c>
     </row>
     <row r="4" spans="1:7" ht="57.95" customHeight="1">
-      <c r="A4" s="33" t="s">
+      <c r="A4" s="41" t="s">
         <v>197</v>
       </c>
-      <c r="B4" s="33" t="s">
+      <c r="B4" s="41" t="s">
         <v>198</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="C4" s="43" t="s">
         <v>199</v>
       </c>
-      <c r="D4" s="29" t="s">
+      <c r="D4" s="43" t="s">
         <v>200</v>
       </c>
-      <c r="E4" s="29" t="s">
+      <c r="E4" s="43" t="s">
         <v>201</v>
       </c>
-      <c r="F4" s="27" t="s">
+      <c r="F4" s="44" t="s">
         <v>202</v>
       </c>
-      <c r="G4" s="27" t="s">
+      <c r="G4" s="44" t="s">
         <v>203</v>
       </c>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="28"/>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
+      <c r="A5" s="42"/>
+      <c r="B5" s="42"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="42"/>
     </row>
     <row r="6" spans="1:7" ht="57.95" customHeight="1">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="43" t="s">
         <v>204</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="43" t="s">
         <v>205</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="43" t="s">
         <v>206</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="43" t="s">
         <v>207</v>
       </c>
-      <c r="E6" s="29" t="s">
+      <c r="E6" s="43" t="s">
         <v>208</v>
       </c>
-      <c r="F6" s="27" t="s">
+      <c r="F6" s="44" t="s">
         <v>209</v>
       </c>
-      <c r="G6" s="27" t="s">
+      <c r="G6" s="44" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="7" spans="1:7">
-      <c r="A7" s="28"/>
-      <c r="B7" s="28"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="28"/>
+      <c r="A7" s="42"/>
+      <c r="B7" s="42"/>
+      <c r="C7" s="42"/>
+      <c r="D7" s="42"/>
+      <c r="E7" s="42"/>
+      <c r="F7" s="42"/>
+      <c r="G7" s="42"/>
     </row>
     <row r="8" spans="1:7" ht="57.95" customHeight="1">
-      <c r="A8" s="29" t="s">
+      <c r="A8" s="43" t="s">
         <v>211</v>
       </c>
-      <c r="B8" s="29" t="s">
+      <c r="B8" s="43" t="s">
         <v>212</v>
       </c>
-      <c r="C8" s="29" t="s">
+      <c r="C8" s="43" t="s">
         <v>213</v>
       </c>
-      <c r="D8" s="29" t="s">
+      <c r="D8" s="43" t="s">
         <v>214</v>
       </c>
-      <c r="E8" s="29" t="s">
+      <c r="E8" s="43" t="s">
         <v>215</v>
       </c>
-      <c r="F8" s="27" t="s">
+      <c r="F8" s="44" t="s">
         <v>216</v>
       </c>
-      <c r="G8" s="27" t="s">
+      <c r="G8" s="44" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="9" spans="1:7">
-      <c r="A9" s="28"/>
-      <c r="B9" s="28"/>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
+      <c r="A9" s="42"/>
+      <c r="B9" s="42"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="42"/>
+      <c r="F9" s="42"/>
+      <c r="G9" s="42"/>
     </row>
     <row r="10" spans="1:7" ht="57.95" customHeight="1">
-      <c r="A10" s="29" t="s">
+      <c r="A10" s="43" t="s">
         <v>218</v>
       </c>
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="43" t="s">
         <v>219</v>
       </c>
-      <c r="C10" s="29" t="s">
+      <c r="C10" s="43" t="s">
         <v>220</v>
       </c>
-      <c r="D10" s="29" t="s">
+      <c r="D10" s="43" t="s">
         <v>221</v>
       </c>
-      <c r="E10" s="29" t="s">
+      <c r="E10" s="43" t="s">
         <v>222</v>
       </c>
-      <c r="F10" s="27" t="s">
+      <c r="F10" s="44" t="s">
         <v>223</v>
       </c>
-      <c r="G10" s="27" t="s">
+      <c r="G10" s="44" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="11" spans="1:7">
-      <c r="A11" s="28"/>
-      <c r="B11" s="28"/>
-      <c r="C11" s="28"/>
-      <c r="D11" s="28"/>
-      <c r="E11" s="28"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="28"/>
+      <c r="A11" s="42"/>
+      <c r="B11" s="42"/>
+      <c r="C11" s="42"/>
+      <c r="D11" s="42"/>
+      <c r="E11" s="42"/>
+      <c r="F11" s="42"/>
+      <c r="G11" s="42"/>
     </row>
     <row r="12" spans="1:7" ht="57.95" customHeight="1">
-      <c r="A12" s="29" t="s">
+      <c r="A12" s="43" t="s">
         <v>225</v>
       </c>
-      <c r="B12" s="29" t="s">
+      <c r="B12" s="43" t="s">
         <v>226</v>
       </c>
-      <c r="C12" s="29" t="s">
+      <c r="C12" s="43" t="s">
         <v>227</v>
       </c>
-      <c r="D12" s="29" t="s">
+      <c r="D12" s="43" t="s">
         <v>228</v>
       </c>
-      <c r="E12" s="33" t="s">
+      <c r="E12" s="41" t="s">
         <v>229</v>
       </c>
-      <c r="F12" s="33" t="s">
+      <c r="F12" s="41" t="s">
         <v>230</v>
       </c>
-      <c r="G12" s="33" t="s">
+      <c r="G12" s="41" t="s">
         <v>231</v>
       </c>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="28"/>
-      <c r="B13" s="28"/>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="28"/>
-      <c r="F13" s="28"/>
-      <c r="G13" s="28"/>
+      <c r="A13" s="42"/>
+      <c r="B13" s="42"/>
+      <c r="C13" s="42"/>
+      <c r="D13" s="42"/>
+      <c r="E13" s="42"/>
+      <c r="F13" s="42"/>
+      <c r="G13" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="36">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="G4:G5"/>
+    <mergeCell ref="F10:F11"/>
+    <mergeCell ref="G10:G11"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="G12:G13"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="E10:E11"/>
     <mergeCell ref="F6:F7"/>
     <mergeCell ref="G6:G7"/>
     <mergeCell ref="A8:A9"/>
@@ -5883,6 +5921,223 @@
     <mergeCell ref="C6:C7"/>
     <mergeCell ref="D6:D7"/>
     <mergeCell ref="E6:E7"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="G4:G5"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="7" width="21" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="24" customHeight="1">
+      <c r="A1" s="29" t="s">
+        <v>232</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="31"/>
+    </row>
+    <row r="3" spans="1:7" ht="15">
+      <c r="A3" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>166</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="F3" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="57.95" customHeight="1">
+      <c r="A4" s="41" t="s">
+        <v>233</v>
+      </c>
+      <c r="B4" s="41" t="s">
+        <v>234</v>
+      </c>
+      <c r="C4" s="41" t="s">
+        <v>235</v>
+      </c>
+      <c r="D4" s="41" t="s">
+        <v>197</v>
+      </c>
+      <c r="E4" s="43" t="s">
+        <v>236</v>
+      </c>
+      <c r="F4" s="44" t="s">
+        <v>237</v>
+      </c>
+      <c r="G4" s="44" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="42"/>
+      <c r="B5" s="42"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="42"/>
+    </row>
+    <row r="6" spans="1:7" ht="57.95" customHeight="1">
+      <c r="A6" s="43" t="s">
+        <v>239</v>
+      </c>
+      <c r="B6" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="C6" s="43" t="s">
+        <v>241</v>
+      </c>
+      <c r="D6" s="43" t="s">
+        <v>242</v>
+      </c>
+      <c r="E6" s="43" t="s">
+        <v>243</v>
+      </c>
+      <c r="F6" s="44" t="s">
+        <v>244</v>
+      </c>
+      <c r="G6" s="44" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="42"/>
+      <c r="B7" s="42"/>
+      <c r="C7" s="42"/>
+      <c r="D7" s="42"/>
+      <c r="E7" s="42"/>
+      <c r="F7" s="42"/>
+      <c r="G7" s="42"/>
+    </row>
+    <row r="8" spans="1:7" ht="57.95" customHeight="1">
+      <c r="A8" s="43" t="s">
+        <v>246</v>
+      </c>
+      <c r="B8" s="43" t="s">
+        <v>247</v>
+      </c>
+      <c r="C8" s="43" t="s">
+        <v>248</v>
+      </c>
+      <c r="D8" s="43" t="s">
+        <v>249</v>
+      </c>
+      <c r="E8" s="43" t="s">
+        <v>250</v>
+      </c>
+      <c r="F8" s="44" t="s">
+        <v>251</v>
+      </c>
+      <c r="G8" s="44" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="42"/>
+      <c r="B9" s="42"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="42"/>
+      <c r="F9" s="42"/>
+      <c r="G9" s="42"/>
+    </row>
+    <row r="10" spans="1:7" ht="57.95" customHeight="1">
+      <c r="A10" s="43" t="s">
+        <v>253</v>
+      </c>
+      <c r="B10" s="43" t="s">
+        <v>254</v>
+      </c>
+      <c r="C10" s="43" t="s">
+        <v>255</v>
+      </c>
+      <c r="D10" s="43" t="s">
+        <v>256</v>
+      </c>
+      <c r="E10" s="43" t="s">
+        <v>257</v>
+      </c>
+      <c r="F10" s="44" t="s">
+        <v>258</v>
+      </c>
+      <c r="G10" s="44" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="42"/>
+      <c r="B11" s="42"/>
+      <c r="C11" s="42"/>
+      <c r="D11" s="42"/>
+      <c r="E11" s="42"/>
+      <c r="F11" s="42"/>
+      <c r="G11" s="42"/>
+    </row>
+    <row r="12" spans="1:7" ht="57.95" customHeight="1">
+      <c r="A12" s="43" t="s">
+        <v>260</v>
+      </c>
+      <c r="B12" s="43" t="s">
+        <v>261</v>
+      </c>
+      <c r="C12" s="43" t="s">
+        <v>262</v>
+      </c>
+      <c r="D12" s="43" t="s">
+        <v>263</v>
+      </c>
+      <c r="E12" s="43" t="s">
+        <v>264</v>
+      </c>
+      <c r="F12" s="44" t="s">
+        <v>265</v>
+      </c>
+      <c r="G12" s="44" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="42"/>
+      <c r="B13" s="42"/>
+      <c r="C13" s="42"/>
+      <c r="D13" s="42"/>
+      <c r="E13" s="42"/>
+      <c r="F13" s="42"/>
+      <c r="G13" s="42"/>
+    </row>
+  </sheetData>
+  <mergeCells count="36">
     <mergeCell ref="F10:F11"/>
     <mergeCell ref="G10:G11"/>
     <mergeCell ref="A12:A13"/>
@@ -5897,223 +6152,6 @@
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="D10:D11"/>
     <mergeCell ref="E10:E11"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
-  <cols>
-    <col min="1" max="7" width="21" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" ht="24" customHeight="1">
-      <c r="A1" s="30" t="s">
-        <v>232</v>
-      </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="32"/>
-    </row>
-    <row r="3" spans="1:7" ht="15">
-      <c r="A3" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>162</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>166</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>170</v>
-      </c>
-      <c r="E3" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="F3" s="14" t="s">
-        <v>195</v>
-      </c>
-      <c r="G3" s="15" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="57.95" customHeight="1">
-      <c r="A4" s="33" t="s">
-        <v>233</v>
-      </c>
-      <c r="B4" s="33" t="s">
-        <v>234</v>
-      </c>
-      <c r="C4" s="33" t="s">
-        <v>235</v>
-      </c>
-      <c r="D4" s="33" t="s">
-        <v>197</v>
-      </c>
-      <c r="E4" s="29" t="s">
-        <v>236</v>
-      </c>
-      <c r="F4" s="27" t="s">
-        <v>237</v>
-      </c>
-      <c r="G4" s="27" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="28"/>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
-    </row>
-    <row r="6" spans="1:7" ht="57.95" customHeight="1">
-      <c r="A6" s="29" t="s">
-        <v>239</v>
-      </c>
-      <c r="B6" s="29" t="s">
-        <v>240</v>
-      </c>
-      <c r="C6" s="29" t="s">
-        <v>241</v>
-      </c>
-      <c r="D6" s="29" t="s">
-        <v>242</v>
-      </c>
-      <c r="E6" s="29" t="s">
-        <v>243</v>
-      </c>
-      <c r="F6" s="27" t="s">
-        <v>244</v>
-      </c>
-      <c r="G6" s="27" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="28"/>
-      <c r="B7" s="28"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="28"/>
-    </row>
-    <row r="8" spans="1:7" ht="57.95" customHeight="1">
-      <c r="A8" s="29" t="s">
-        <v>246</v>
-      </c>
-      <c r="B8" s="29" t="s">
-        <v>247</v>
-      </c>
-      <c r="C8" s="29" t="s">
-        <v>248</v>
-      </c>
-      <c r="D8" s="29" t="s">
-        <v>249</v>
-      </c>
-      <c r="E8" s="29" t="s">
-        <v>250</v>
-      </c>
-      <c r="F8" s="27" t="s">
-        <v>251</v>
-      </c>
-      <c r="G8" s="27" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="28"/>
-      <c r="B9" s="28"/>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-    </row>
-    <row r="10" spans="1:7" ht="57.95" customHeight="1">
-      <c r="A10" s="29" t="s">
-        <v>253</v>
-      </c>
-      <c r="B10" s="29" t="s">
-        <v>254</v>
-      </c>
-      <c r="C10" s="29" t="s">
-        <v>255</v>
-      </c>
-      <c r="D10" s="29" t="s">
-        <v>256</v>
-      </c>
-      <c r="E10" s="29" t="s">
-        <v>257</v>
-      </c>
-      <c r="F10" s="27" t="s">
-        <v>258</v>
-      </c>
-      <c r="G10" s="27" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="28"/>
-      <c r="B11" s="28"/>
-      <c r="C11" s="28"/>
-      <c r="D11" s="28"/>
-      <c r="E11" s="28"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="28"/>
-    </row>
-    <row r="12" spans="1:7" ht="57.95" customHeight="1">
-      <c r="A12" s="29" t="s">
-        <v>260</v>
-      </c>
-      <c r="B12" s="29" t="s">
-        <v>261</v>
-      </c>
-      <c r="C12" s="29" t="s">
-        <v>262</v>
-      </c>
-      <c r="D12" s="29" t="s">
-        <v>263</v>
-      </c>
-      <c r="E12" s="29" t="s">
-        <v>264</v>
-      </c>
-      <c r="F12" s="27" t="s">
-        <v>265</v>
-      </c>
-      <c r="G12" s="27" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13" s="28"/>
-      <c r="B13" s="28"/>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="28"/>
-      <c r="F13" s="28"/>
-      <c r="G13" s="28"/>
-    </row>
-  </sheetData>
-  <mergeCells count="36">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="G4:G5"/>
     <mergeCell ref="F6:F7"/>
     <mergeCell ref="G6:G7"/>
     <mergeCell ref="A8:A9"/>
@@ -6128,20 +6166,14 @@
     <mergeCell ref="C6:C7"/>
     <mergeCell ref="D6:D7"/>
     <mergeCell ref="E6:E7"/>
-    <mergeCell ref="F10:F11"/>
-    <mergeCell ref="G10:G11"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="F12:F13"/>
-    <mergeCell ref="G12:G13"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="G4:G5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>